<commit_message>
Update results template Excel files
Replace/update multiple binary .xlsx result templates across benchmark sets. Affected files include dimension-specific templates (10/15/20/30/50/100Dim) and fixDim files for CEC2005, CEC2014, CEC2017, CEC2019, CEC2020, CEC2022 and Real World Problems. These updates adjust the spreadsheet templates (formatting/dimensions/content) used for results output; no source code changes.
</commit_message>
<xml_diff>
--- a/src/results_template/CEC2014/10Dim.xlsx
+++ b/src/results_template/CEC2014/10Dim.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GtiHub\Repositories\Base-Optimization-Framework\src\results\results_template\CEC2014\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GtiHub\Repositories\Base-Optimization-Framework\src\results_template\CEC2014\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A3567B-1AD7-4558-9C04-2D45119370D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE2C57A-2A7B-4BC9-9CB5-376CE7AF99B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conclusions" sheetId="2" r:id="rId1"/>
@@ -34,8 +34,33 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2107,65 +2132,65 @@
       <c r="T3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V3" s="7" t="e">
-        <f t="shared" ref="V3:AJ3" si="1">_xlfn.RANK.EQ(D3,$D3:$R3,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ3" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
+      <c r="V3" s="7" t="e" cm="1">
+        <f t="array" ref="V3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(D3,2-INT(LOG10(ABS(D3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W3" s="7" t="e" cm="1">
+        <f t="array" ref="W3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(E3,2-INT(LOG10(ABS(E3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X3" s="7" t="e" cm="1">
+        <f t="array" ref="X3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(F3,2-INT(LOG10(ABS(F3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y3" s="7" t="e" cm="1">
+        <f t="array" ref="Y3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(G3,2-INT(LOG10(ABS(G3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z3" s="7" t="e" cm="1">
+        <f t="array" ref="Z3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(H3,2-INT(LOG10(ABS(H3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA3" s="7" t="e" cm="1">
+        <f t="array" ref="AA3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(I3,2-INT(LOG10(ABS(I3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB3" s="7" t="e" cm="1">
+        <f t="array" ref="AB3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(J3,2-INT(LOG10(ABS(J3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC3" s="7" t="e" cm="1">
+        <f t="array" ref="AC3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(K3,2-INT(LOG10(ABS(K3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD3" s="7" t="e" cm="1">
+        <f t="array" ref="AD3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(L3,2-INT(LOG10(ABS(L3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE3" s="7" t="e" cm="1">
+        <f t="array" ref="AE3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(M3,2-INT(LOG10(ABS(M3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF3" s="7" t="e" cm="1">
+        <f t="array" ref="AF3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(N3,2-INT(LOG10(ABS(N3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG3" s="7" t="e" cm="1">
+        <f t="array" ref="AG3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(O3,2-INT(LOG10(ABS(O3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH3" s="7" t="e" cm="1">
+        <f t="array" ref="AH3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(P3,2-INT(LOG10(ABS(P3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI3" s="7" t="e" cm="1">
+        <f t="array" ref="AI3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(Q3,2-INT(LOG10(ABS(Q3))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ3" s="7" t="e" cm="1">
+        <f t="array" ref="AJ3">SUMPRODUCT(--(ROUND($D3:$R3,2-INT(LOG10(ABS($D3:$R3))))&lt;ROUND(R3,2-INT(LOG10(ABS(R3))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
@@ -2275,65 +2300,65 @@
       <c r="T6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="7" t="e">
-        <f t="shared" ref="V6:AJ6" si="2">_xlfn.RANK.EQ(D6,$D6:$R6,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ6" s="7" t="e">
-        <f t="shared" si="2"/>
-        <v>#N/A</v>
+      <c r="V6" s="7" t="e" cm="1">
+        <f t="array" ref="V6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(D6,2-INT(LOG10(ABS(D6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W6" s="7" t="e" cm="1">
+        <f t="array" ref="W6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(E6,2-INT(LOG10(ABS(E6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X6" s="7" t="e" cm="1">
+        <f t="array" ref="X6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(F6,2-INT(LOG10(ABS(F6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y6" s="7" t="e" cm="1">
+        <f t="array" ref="Y6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(G6,2-INT(LOG10(ABS(G6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z6" s="7" t="e" cm="1">
+        <f t="array" ref="Z6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(H6,2-INT(LOG10(ABS(H6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA6" s="7" t="e" cm="1">
+        <f t="array" ref="AA6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(I6,2-INT(LOG10(ABS(I6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB6" s="7" t="e" cm="1">
+        <f t="array" ref="AB6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(J6,2-INT(LOG10(ABS(J6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC6" s="7" t="e" cm="1">
+        <f t="array" ref="AC6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(K6,2-INT(LOG10(ABS(K6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD6" s="7" t="e" cm="1">
+        <f t="array" ref="AD6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(L6,2-INT(LOG10(ABS(L6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE6" s="7" t="e" cm="1">
+        <f t="array" ref="AE6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(M6,2-INT(LOG10(ABS(M6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF6" s="7" t="e" cm="1">
+        <f t="array" ref="AF6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(N6,2-INT(LOG10(ABS(N6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG6" s="7" t="e" cm="1">
+        <f t="array" ref="AG6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(O6,2-INT(LOG10(ABS(O6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH6" s="7" t="e" cm="1">
+        <f t="array" ref="AH6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(P6,2-INT(LOG10(ABS(P6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI6" s="7" t="e" cm="1">
+        <f t="array" ref="AI6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(Q6,2-INT(LOG10(ABS(Q6))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ6" s="7" t="e" cm="1">
+        <f t="array" ref="AJ6">SUMPRODUCT(--(ROUND($D6:$R6,2-INT(LOG10(ABS($D6:$R6))))&lt;ROUND(R6,2-INT(LOG10(ABS(R6))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
@@ -2443,65 +2468,65 @@
       <c r="T9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V9" s="7" t="e">
-        <f t="shared" ref="V9:AJ9" si="3">_xlfn.RANK.EQ(D9,$D9:$R9,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ9" s="7" t="e">
-        <f t="shared" si="3"/>
-        <v>#N/A</v>
+      <c r="V9" s="7" t="e" cm="1">
+        <f t="array" ref="V9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(D9,2-INT(LOG10(ABS(D9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W9" s="7" t="e" cm="1">
+        <f t="array" ref="W9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(E9,2-INT(LOG10(ABS(E9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X9" s="7" t="e" cm="1">
+        <f t="array" ref="X9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(F9,2-INT(LOG10(ABS(F9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y9" s="7" t="e" cm="1">
+        <f t="array" ref="Y9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(G9,2-INT(LOG10(ABS(G9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z9" s="7" t="e" cm="1">
+        <f t="array" ref="Z9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(H9,2-INT(LOG10(ABS(H9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA9" s="7" t="e" cm="1">
+        <f t="array" ref="AA9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(I9,2-INT(LOG10(ABS(I9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB9" s="7" t="e" cm="1">
+        <f t="array" ref="AB9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(J9,2-INT(LOG10(ABS(J9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC9" s="7" t="e" cm="1">
+        <f t="array" ref="AC9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(K9,2-INT(LOG10(ABS(K9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD9" s="7" t="e" cm="1">
+        <f t="array" ref="AD9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(L9,2-INT(LOG10(ABS(L9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE9" s="7" t="e" cm="1">
+        <f t="array" ref="AE9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(M9,2-INT(LOG10(ABS(M9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF9" s="7" t="e" cm="1">
+        <f t="array" ref="AF9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(N9,2-INT(LOG10(ABS(N9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG9" s="7" t="e" cm="1">
+        <f t="array" ref="AG9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(O9,2-INT(LOG10(ABS(O9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH9" s="7" t="e" cm="1">
+        <f t="array" ref="AH9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(P9,2-INT(LOG10(ABS(P9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI9" s="7" t="e" cm="1">
+        <f t="array" ref="AI9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(Q9,2-INT(LOG10(ABS(Q9))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ9" s="7" t="e" cm="1">
+        <f t="array" ref="AJ9">SUMPRODUCT(--(ROUND($D9:$R9,2-INT(LOG10(ABS($D9:$R9))))&lt;ROUND(R9,2-INT(LOG10(ABS(R9))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="10" spans="1:36" x14ac:dyDescent="0.25">
@@ -2613,65 +2638,65 @@
       <c r="T12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V12" s="7" t="e">
-        <f t="shared" ref="V12:AJ12" si="4">_xlfn.RANK.EQ(D12,$D12:$R12,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ12" s="7" t="e">
-        <f t="shared" si="4"/>
-        <v>#N/A</v>
+      <c r="V12" s="7" t="e" cm="1">
+        <f t="array" ref="V12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(D12,2-INT(LOG10(ABS(D12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W12" s="7" t="e" cm="1">
+        <f t="array" ref="W12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(E12,2-INT(LOG10(ABS(E12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X12" s="7" t="e" cm="1">
+        <f t="array" ref="X12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(F12,2-INT(LOG10(ABS(F12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y12" s="7" t="e" cm="1">
+        <f t="array" ref="Y12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(G12,2-INT(LOG10(ABS(G12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z12" s="7" t="e" cm="1">
+        <f t="array" ref="Z12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(H12,2-INT(LOG10(ABS(H12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA12" s="7" t="e" cm="1">
+        <f t="array" ref="AA12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(I12,2-INT(LOG10(ABS(I12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB12" s="7" t="e" cm="1">
+        <f t="array" ref="AB12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(J12,2-INT(LOG10(ABS(J12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC12" s="7" t="e" cm="1">
+        <f t="array" ref="AC12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(K12,2-INT(LOG10(ABS(K12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD12" s="7" t="e" cm="1">
+        <f t="array" ref="AD12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(L12,2-INT(LOG10(ABS(L12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE12" s="7" t="e" cm="1">
+        <f t="array" ref="AE12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(M12,2-INT(LOG10(ABS(M12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF12" s="7" t="e" cm="1">
+        <f t="array" ref="AF12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(N12,2-INT(LOG10(ABS(N12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG12" s="7" t="e" cm="1">
+        <f t="array" ref="AG12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(O12,2-INT(LOG10(ABS(O12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH12" s="7" t="e" cm="1">
+        <f t="array" ref="AH12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(P12,2-INT(LOG10(ABS(P12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI12" s="7" t="e" cm="1">
+        <f t="array" ref="AI12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(Q12,2-INT(LOG10(ABS(Q12))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ12" s="7" t="e" cm="1">
+        <f t="array" ref="AJ12">SUMPRODUCT(--(ROUND($D12:$R12,2-INT(LOG10(ABS($D12:$R12))))&lt;ROUND(R12,2-INT(LOG10(ABS(R12))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -2781,65 +2806,65 @@
       <c r="T15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V15" s="7" t="e">
-        <f t="shared" ref="V15:AJ15" si="5">_xlfn.RANK.EQ(D15,$D15:$R15,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ15" s="7" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
+      <c r="V15" s="7" t="e" cm="1">
+        <f t="array" ref="V15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(D15,2-INT(LOG10(ABS(D15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W15" s="7" t="e" cm="1">
+        <f t="array" ref="W15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(E15,2-INT(LOG10(ABS(E15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X15" s="7" t="e" cm="1">
+        <f t="array" ref="X15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(F15,2-INT(LOG10(ABS(F15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y15" s="7" t="e" cm="1">
+        <f t="array" ref="Y15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(G15,2-INT(LOG10(ABS(G15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z15" s="7" t="e" cm="1">
+        <f t="array" ref="Z15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(H15,2-INT(LOG10(ABS(H15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA15" s="7" t="e" cm="1">
+        <f t="array" ref="AA15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(I15,2-INT(LOG10(ABS(I15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB15" s="7" t="e" cm="1">
+        <f t="array" ref="AB15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(J15,2-INT(LOG10(ABS(J15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC15" s="7" t="e" cm="1">
+        <f t="array" ref="AC15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(K15,2-INT(LOG10(ABS(K15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD15" s="7" t="e" cm="1">
+        <f t="array" ref="AD15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(L15,2-INT(LOG10(ABS(L15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE15" s="7" t="e" cm="1">
+        <f t="array" ref="AE15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(M15,2-INT(LOG10(ABS(M15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF15" s="7" t="e" cm="1">
+        <f t="array" ref="AF15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(N15,2-INT(LOG10(ABS(N15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG15" s="7" t="e" cm="1">
+        <f t="array" ref="AG15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(O15,2-INT(LOG10(ABS(O15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH15" s="7" t="e" cm="1">
+        <f t="array" ref="AH15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(P15,2-INT(LOG10(ABS(P15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI15" s="7" t="e" cm="1">
+        <f t="array" ref="AI15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(Q15,2-INT(LOG10(ABS(Q15))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ15" s="7" t="e" cm="1">
+        <f t="array" ref="AJ15">SUMPRODUCT(--(ROUND($D15:$R15,2-INT(LOG10(ABS($D15:$R15))))&lt;ROUND(R15,2-INT(LOG10(ABS(R15))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="16" spans="1:36" x14ac:dyDescent="0.25">
@@ -2949,65 +2974,65 @@
       <c r="T18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V18" s="7" t="e">
-        <f t="shared" ref="V18:AJ18" si="6">_xlfn.RANK.EQ(D18,$D18:$R18,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ18" s="7" t="e">
-        <f t="shared" si="6"/>
-        <v>#N/A</v>
+      <c r="V18" s="7" t="e" cm="1">
+        <f t="array" ref="V18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(D18,2-INT(LOG10(ABS(D18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W18" s="7" t="e" cm="1">
+        <f t="array" ref="W18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(E18,2-INT(LOG10(ABS(E18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X18" s="7" t="e" cm="1">
+        <f t="array" ref="X18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(F18,2-INT(LOG10(ABS(F18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y18" s="7" t="e" cm="1">
+        <f t="array" ref="Y18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(G18,2-INT(LOG10(ABS(G18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z18" s="7" t="e" cm="1">
+        <f t="array" ref="Z18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(H18,2-INT(LOG10(ABS(H18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA18" s="7" t="e" cm="1">
+        <f t="array" ref="AA18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(I18,2-INT(LOG10(ABS(I18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB18" s="7" t="e" cm="1">
+        <f t="array" ref="AB18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(J18,2-INT(LOG10(ABS(J18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC18" s="7" t="e" cm="1">
+        <f t="array" ref="AC18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(K18,2-INT(LOG10(ABS(K18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD18" s="7" t="e" cm="1">
+        <f t="array" ref="AD18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(L18,2-INT(LOG10(ABS(L18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE18" s="7" t="e" cm="1">
+        <f t="array" ref="AE18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(M18,2-INT(LOG10(ABS(M18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF18" s="7" t="e" cm="1">
+        <f t="array" ref="AF18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(N18,2-INT(LOG10(ABS(N18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG18" s="7" t="e" cm="1">
+        <f t="array" ref="AG18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(O18,2-INT(LOG10(ABS(O18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH18" s="7" t="e" cm="1">
+        <f t="array" ref="AH18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(P18,2-INT(LOG10(ABS(P18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI18" s="7" t="e" cm="1">
+        <f t="array" ref="AI18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(Q18,2-INT(LOG10(ABS(Q18))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ18" s="7" t="e" cm="1">
+        <f t="array" ref="AJ18">SUMPRODUCT(--(ROUND($D18:$R18,2-INT(LOG10(ABS($D18:$R18))))&lt;ROUND(R18,2-INT(LOG10(ABS(R18))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="19" spans="1:36" x14ac:dyDescent="0.25">
@@ -3117,65 +3142,65 @@
       <c r="T21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V21" s="7" t="e">
-        <f t="shared" ref="V21:AJ21" si="7">_xlfn.RANK.EQ(D21,$D21:$R21,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ21" s="7" t="e">
-        <f t="shared" si="7"/>
-        <v>#N/A</v>
+      <c r="V21" s="7" t="e" cm="1">
+        <f t="array" ref="V21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(D21,2-INT(LOG10(ABS(D21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W21" s="7" t="e" cm="1">
+        <f t="array" ref="W21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(E21,2-INT(LOG10(ABS(E21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X21" s="7" t="e" cm="1">
+        <f t="array" ref="X21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(F21,2-INT(LOG10(ABS(F21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y21" s="7" t="e" cm="1">
+        <f t="array" ref="Y21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(G21,2-INT(LOG10(ABS(G21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z21" s="7" t="e" cm="1">
+        <f t="array" ref="Z21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(H21,2-INT(LOG10(ABS(H21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA21" s="7" t="e" cm="1">
+        <f t="array" ref="AA21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(I21,2-INT(LOG10(ABS(I21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB21" s="7" t="e" cm="1">
+        <f t="array" ref="AB21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(J21,2-INT(LOG10(ABS(J21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC21" s="7" t="e" cm="1">
+        <f t="array" ref="AC21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(K21,2-INT(LOG10(ABS(K21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD21" s="7" t="e" cm="1">
+        <f t="array" ref="AD21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(L21,2-INT(LOG10(ABS(L21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE21" s="7" t="e" cm="1">
+        <f t="array" ref="AE21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(M21,2-INT(LOG10(ABS(M21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF21" s="7" t="e" cm="1">
+        <f t="array" ref="AF21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(N21,2-INT(LOG10(ABS(N21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG21" s="7" t="e" cm="1">
+        <f t="array" ref="AG21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(O21,2-INT(LOG10(ABS(O21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH21" s="7" t="e" cm="1">
+        <f t="array" ref="AH21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(P21,2-INT(LOG10(ABS(P21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI21" s="7" t="e" cm="1">
+        <f t="array" ref="AI21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(Q21,2-INT(LOG10(ABS(Q21))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ21" s="7" t="e" cm="1">
+        <f t="array" ref="AJ21">SUMPRODUCT(--(ROUND($D21:$R21,2-INT(LOG10(ABS($D21:$R21))))&lt;ROUND(R21,2-INT(LOG10(ABS(R21))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="22" spans="1:36" x14ac:dyDescent="0.25">
@@ -3285,65 +3310,65 @@
       <c r="T24" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V24" s="7" t="e">
-        <f t="shared" ref="V24:AJ24" si="8">_xlfn.RANK.EQ(D24,$D24:$R24,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ24" s="7" t="e">
-        <f t="shared" si="8"/>
-        <v>#N/A</v>
+      <c r="V24" s="7" t="e" cm="1">
+        <f t="array" ref="V24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(D24,2-INT(LOG10(ABS(D24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W24" s="7" t="e" cm="1">
+        <f t="array" ref="W24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(E24,2-INT(LOG10(ABS(E24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X24" s="7" t="e" cm="1">
+        <f t="array" ref="X24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(F24,2-INT(LOG10(ABS(F24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y24" s="7" t="e" cm="1">
+        <f t="array" ref="Y24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(G24,2-INT(LOG10(ABS(G24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z24" s="7" t="e" cm="1">
+        <f t="array" ref="Z24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(H24,2-INT(LOG10(ABS(H24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA24" s="7" t="e" cm="1">
+        <f t="array" ref="AA24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(I24,2-INT(LOG10(ABS(I24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB24" s="7" t="e" cm="1">
+        <f t="array" ref="AB24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(J24,2-INT(LOG10(ABS(J24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC24" s="7" t="e" cm="1">
+        <f t="array" ref="AC24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(K24,2-INT(LOG10(ABS(K24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD24" s="7" t="e" cm="1">
+        <f t="array" ref="AD24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(L24,2-INT(LOG10(ABS(L24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE24" s="7" t="e" cm="1">
+        <f t="array" ref="AE24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(M24,2-INT(LOG10(ABS(M24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF24" s="7" t="e" cm="1">
+        <f t="array" ref="AF24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(N24,2-INT(LOG10(ABS(N24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG24" s="7" t="e" cm="1">
+        <f t="array" ref="AG24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(O24,2-INT(LOG10(ABS(O24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH24" s="7" t="e" cm="1">
+        <f t="array" ref="AH24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(P24,2-INT(LOG10(ABS(P24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI24" s="7" t="e" cm="1">
+        <f t="array" ref="AI24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(Q24,2-INT(LOG10(ABS(Q24))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ24" s="7" t="e" cm="1">
+        <f t="array" ref="AJ24">SUMPRODUCT(--(ROUND($D24:$R24,2-INT(LOG10(ABS($D24:$R24))))&lt;ROUND(R24,2-INT(LOG10(ABS(R24))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="25" spans="1:36" x14ac:dyDescent="0.25">
@@ -3453,65 +3478,65 @@
       <c r="T27" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V27" s="7" t="e">
-        <f t="shared" ref="V27:AJ27" si="9">_xlfn.RANK.EQ(D27,$D27:$R27,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ27" s="7" t="e">
-        <f t="shared" si="9"/>
-        <v>#N/A</v>
+      <c r="V27" s="7" t="e" cm="1">
+        <f t="array" ref="V27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(D27,2-INT(LOG10(ABS(D27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W27" s="7" t="e" cm="1">
+        <f t="array" ref="W27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(E27,2-INT(LOG10(ABS(E27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X27" s="7" t="e" cm="1">
+        <f t="array" ref="X27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(F27,2-INT(LOG10(ABS(F27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y27" s="7" t="e" cm="1">
+        <f t="array" ref="Y27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(G27,2-INT(LOG10(ABS(G27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z27" s="7" t="e" cm="1">
+        <f t="array" ref="Z27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(H27,2-INT(LOG10(ABS(H27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA27" s="7" t="e" cm="1">
+        <f t="array" ref="AA27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(I27,2-INT(LOG10(ABS(I27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB27" s="7" t="e" cm="1">
+        <f t="array" ref="AB27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(J27,2-INT(LOG10(ABS(J27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC27" s="7" t="e" cm="1">
+        <f t="array" ref="AC27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(K27,2-INT(LOG10(ABS(K27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD27" s="7" t="e" cm="1">
+        <f t="array" ref="AD27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(L27,2-INT(LOG10(ABS(L27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE27" s="7" t="e" cm="1">
+        <f t="array" ref="AE27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(M27,2-INT(LOG10(ABS(M27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF27" s="7" t="e" cm="1">
+        <f t="array" ref="AF27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(N27,2-INT(LOG10(ABS(N27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG27" s="7" t="e" cm="1">
+        <f t="array" ref="AG27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(O27,2-INT(LOG10(ABS(O27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH27" s="7" t="e" cm="1">
+        <f t="array" ref="AH27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(P27,2-INT(LOG10(ABS(P27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI27" s="7" t="e" cm="1">
+        <f t="array" ref="AI27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(Q27,2-INT(LOG10(ABS(Q27))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ27" s="7" t="e" cm="1">
+        <f t="array" ref="AJ27">SUMPRODUCT(--(ROUND($D27:$R27,2-INT(LOG10(ABS($D27:$R27))))&lt;ROUND(R27,2-INT(LOG10(ABS(R27))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="28" spans="1:36" x14ac:dyDescent="0.25">
@@ -3621,65 +3646,65 @@
       <c r="T30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V30" s="7" t="e">
-        <f t="shared" ref="V30:AJ30" si="10">_xlfn.RANK.EQ(D30,$D30:$R30,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ30" s="7" t="e">
-        <f t="shared" si="10"/>
-        <v>#N/A</v>
+      <c r="V30" s="7" t="e" cm="1">
+        <f t="array" ref="V30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(D30,2-INT(LOG10(ABS(D30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W30" s="7" t="e" cm="1">
+        <f t="array" ref="W30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(E30,2-INT(LOG10(ABS(E30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X30" s="7" t="e" cm="1">
+        <f t="array" ref="X30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(F30,2-INT(LOG10(ABS(F30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y30" s="7" t="e" cm="1">
+        <f t="array" ref="Y30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(G30,2-INT(LOG10(ABS(G30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z30" s="7" t="e" cm="1">
+        <f t="array" ref="Z30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(H30,2-INT(LOG10(ABS(H30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA30" s="7" t="e" cm="1">
+        <f t="array" ref="AA30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(I30,2-INT(LOG10(ABS(I30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB30" s="7" t="e" cm="1">
+        <f t="array" ref="AB30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(J30,2-INT(LOG10(ABS(J30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC30" s="7" t="e" cm="1">
+        <f t="array" ref="AC30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(K30,2-INT(LOG10(ABS(K30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD30" s="7" t="e" cm="1">
+        <f t="array" ref="AD30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(L30,2-INT(LOG10(ABS(L30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE30" s="7" t="e" cm="1">
+        <f t="array" ref="AE30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(M30,2-INT(LOG10(ABS(M30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF30" s="7" t="e" cm="1">
+        <f t="array" ref="AF30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(N30,2-INT(LOG10(ABS(N30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG30" s="7" t="e" cm="1">
+        <f t="array" ref="AG30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(O30,2-INT(LOG10(ABS(O30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH30" s="7" t="e" cm="1">
+        <f t="array" ref="AH30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(P30,2-INT(LOG10(ABS(P30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI30" s="7" t="e" cm="1">
+        <f t="array" ref="AI30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(Q30,2-INT(LOG10(ABS(Q30))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ30" s="7" t="e" cm="1">
+        <f t="array" ref="AJ30">SUMPRODUCT(--(ROUND($D30:$R30,2-INT(LOG10(ABS($D30:$R30))))&lt;ROUND(R30,2-INT(LOG10(ABS(R30))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="31" spans="1:36" x14ac:dyDescent="0.25">
@@ -3789,65 +3814,65 @@
       <c r="T33" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V33" s="7" t="e">
-        <f t="shared" ref="V33:AJ33" si="11">_xlfn.RANK.EQ(D33,$D33:$R33,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ33" s="7" t="e">
-        <f t="shared" si="11"/>
-        <v>#N/A</v>
+      <c r="V33" s="7" t="e" cm="1">
+        <f t="array" ref="V33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(D33,2-INT(LOG10(ABS(D33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W33" s="7" t="e" cm="1">
+        <f t="array" ref="W33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(E33,2-INT(LOG10(ABS(E33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X33" s="7" t="e" cm="1">
+        <f t="array" ref="X33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(F33,2-INT(LOG10(ABS(F33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y33" s="7" t="e" cm="1">
+        <f t="array" ref="Y33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(G33,2-INT(LOG10(ABS(G33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z33" s="7" t="e" cm="1">
+        <f t="array" ref="Z33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(H33,2-INT(LOG10(ABS(H33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA33" s="7" t="e" cm="1">
+        <f t="array" ref="AA33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(I33,2-INT(LOG10(ABS(I33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB33" s="7" t="e" cm="1">
+        <f t="array" ref="AB33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(J33,2-INT(LOG10(ABS(J33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC33" s="7" t="e" cm="1">
+        <f t="array" ref="AC33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(K33,2-INT(LOG10(ABS(K33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD33" s="7" t="e" cm="1">
+        <f t="array" ref="AD33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(L33,2-INT(LOG10(ABS(L33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE33" s="7" t="e" cm="1">
+        <f t="array" ref="AE33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(M33,2-INT(LOG10(ABS(M33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF33" s="7" t="e" cm="1">
+        <f t="array" ref="AF33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(N33,2-INT(LOG10(ABS(N33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG33" s="7" t="e" cm="1">
+        <f t="array" ref="AG33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(O33,2-INT(LOG10(ABS(O33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH33" s="7" t="e" cm="1">
+        <f t="array" ref="AH33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(P33,2-INT(LOG10(ABS(P33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI33" s="7" t="e" cm="1">
+        <f t="array" ref="AI33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(Q33,2-INT(LOG10(ABS(Q33))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ33" s="7" t="e" cm="1">
+        <f t="array" ref="AJ33">SUMPRODUCT(--(ROUND($D33:$R33,2-INT(LOG10(ABS($D33:$R33))))&lt;ROUND(R33,2-INT(LOG10(ABS(R33))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="34" spans="1:36" x14ac:dyDescent="0.25">
@@ -3957,65 +3982,65 @@
       <c r="T36" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V36" s="7" t="e">
-        <f t="shared" ref="V36:AJ36" si="12">_xlfn.RANK.EQ(D36,$D36:$R36,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ36" s="7" t="e">
-        <f t="shared" si="12"/>
-        <v>#N/A</v>
+      <c r="V36" s="7" t="e" cm="1">
+        <f t="array" ref="V36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(D36,2-INT(LOG10(ABS(D36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W36" s="7" t="e" cm="1">
+        <f t="array" ref="W36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(E36,2-INT(LOG10(ABS(E36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X36" s="7" t="e" cm="1">
+        <f t="array" ref="X36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(F36,2-INT(LOG10(ABS(F36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y36" s="7" t="e" cm="1">
+        <f t="array" ref="Y36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(G36,2-INT(LOG10(ABS(G36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z36" s="7" t="e" cm="1">
+        <f t="array" ref="Z36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(H36,2-INT(LOG10(ABS(H36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA36" s="7" t="e" cm="1">
+        <f t="array" ref="AA36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(I36,2-INT(LOG10(ABS(I36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB36" s="7" t="e" cm="1">
+        <f t="array" ref="AB36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(J36,2-INT(LOG10(ABS(J36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC36" s="7" t="e" cm="1">
+        <f t="array" ref="AC36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(K36,2-INT(LOG10(ABS(K36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD36" s="7" t="e" cm="1">
+        <f t="array" ref="AD36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(L36,2-INT(LOG10(ABS(L36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE36" s="7" t="e" cm="1">
+        <f t="array" ref="AE36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(M36,2-INT(LOG10(ABS(M36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF36" s="7" t="e" cm="1">
+        <f t="array" ref="AF36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(N36,2-INT(LOG10(ABS(N36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG36" s="7" t="e" cm="1">
+        <f t="array" ref="AG36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(O36,2-INT(LOG10(ABS(O36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH36" s="7" t="e" cm="1">
+        <f t="array" ref="AH36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(P36,2-INT(LOG10(ABS(P36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI36" s="7" t="e" cm="1">
+        <f t="array" ref="AI36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(Q36,2-INT(LOG10(ABS(Q36))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ36" s="7" t="e" cm="1">
+        <f t="array" ref="AJ36">SUMPRODUCT(--(ROUND($D36:$R36,2-INT(LOG10(ABS($D36:$R36))))&lt;ROUND(R36,2-INT(LOG10(ABS(R36))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="37" spans="1:36" x14ac:dyDescent="0.25">
@@ -4125,65 +4150,65 @@
       <c r="T39" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V39" s="7" t="e">
-        <f t="shared" ref="V39:AJ39" si="13">_xlfn.RANK.EQ(D39,$D39:$R39,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ39" s="7" t="e">
-        <f t="shared" si="13"/>
-        <v>#N/A</v>
+      <c r="V39" s="7" t="e" cm="1">
+        <f t="array" ref="V39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(D39,2-INT(LOG10(ABS(D39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W39" s="7" t="e" cm="1">
+        <f t="array" ref="W39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(E39,2-INT(LOG10(ABS(E39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X39" s="7" t="e" cm="1">
+        <f t="array" ref="X39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(F39,2-INT(LOG10(ABS(F39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y39" s="7" t="e" cm="1">
+        <f t="array" ref="Y39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(G39,2-INT(LOG10(ABS(G39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z39" s="7" t="e" cm="1">
+        <f t="array" ref="Z39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(H39,2-INT(LOG10(ABS(H39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA39" s="7" t="e" cm="1">
+        <f t="array" ref="AA39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(I39,2-INT(LOG10(ABS(I39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB39" s="7" t="e" cm="1">
+        <f t="array" ref="AB39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(J39,2-INT(LOG10(ABS(J39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC39" s="7" t="e" cm="1">
+        <f t="array" ref="AC39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(K39,2-INT(LOG10(ABS(K39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD39" s="7" t="e" cm="1">
+        <f t="array" ref="AD39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(L39,2-INT(LOG10(ABS(L39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE39" s="7" t="e" cm="1">
+        <f t="array" ref="AE39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(M39,2-INT(LOG10(ABS(M39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF39" s="7" t="e" cm="1">
+        <f t="array" ref="AF39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(N39,2-INT(LOG10(ABS(N39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG39" s="7" t="e" cm="1">
+        <f t="array" ref="AG39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(O39,2-INT(LOG10(ABS(O39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH39" s="7" t="e" cm="1">
+        <f t="array" ref="AH39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(P39,2-INT(LOG10(ABS(P39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI39" s="7" t="e" cm="1">
+        <f t="array" ref="AI39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(Q39,2-INT(LOG10(ABS(Q39))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ39" s="7" t="e" cm="1">
+        <f t="array" ref="AJ39">SUMPRODUCT(--(ROUND($D39:$R39,2-INT(LOG10(ABS($D39:$R39))))&lt;ROUND(R39,2-INT(LOG10(ABS(R39))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="40" spans="1:36" x14ac:dyDescent="0.25">
@@ -4293,65 +4318,65 @@
       <c r="T42" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V42" s="7" t="e">
-        <f t="shared" ref="V42:AJ42" si="14">_xlfn.RANK.EQ(D42,$D42:$R42,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ42" s="7" t="e">
-        <f t="shared" si="14"/>
-        <v>#N/A</v>
+      <c r="V42" s="7" t="e" cm="1">
+        <f t="array" ref="V42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(D42,2-INT(LOG10(ABS(D42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W42" s="7" t="e" cm="1">
+        <f t="array" ref="W42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(E42,2-INT(LOG10(ABS(E42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X42" s="7" t="e" cm="1">
+        <f t="array" ref="X42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(F42,2-INT(LOG10(ABS(F42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y42" s="7" t="e" cm="1">
+        <f t="array" ref="Y42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(G42,2-INT(LOG10(ABS(G42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z42" s="7" t="e" cm="1">
+        <f t="array" ref="Z42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(H42,2-INT(LOG10(ABS(H42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA42" s="7" t="e" cm="1">
+        <f t="array" ref="AA42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(I42,2-INT(LOG10(ABS(I42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB42" s="7" t="e" cm="1">
+        <f t="array" ref="AB42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(J42,2-INT(LOG10(ABS(J42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC42" s="7" t="e" cm="1">
+        <f t="array" ref="AC42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(K42,2-INT(LOG10(ABS(K42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD42" s="7" t="e" cm="1">
+        <f t="array" ref="AD42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(L42,2-INT(LOG10(ABS(L42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE42" s="7" t="e" cm="1">
+        <f t="array" ref="AE42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(M42,2-INT(LOG10(ABS(M42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF42" s="7" t="e" cm="1">
+        <f t="array" ref="AF42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(N42,2-INT(LOG10(ABS(N42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG42" s="7" t="e" cm="1">
+        <f t="array" ref="AG42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(O42,2-INT(LOG10(ABS(O42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH42" s="7" t="e" cm="1">
+        <f t="array" ref="AH42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(P42,2-INT(LOG10(ABS(P42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI42" s="7" t="e" cm="1">
+        <f t="array" ref="AI42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(Q42,2-INT(LOG10(ABS(Q42))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ42" s="7" t="e" cm="1">
+        <f t="array" ref="AJ42">SUMPRODUCT(--(ROUND($D42:$R42,2-INT(LOG10(ABS($D42:$R42))))&lt;ROUND(R42,2-INT(LOG10(ABS(R42))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="43" spans="1:36" x14ac:dyDescent="0.25">
@@ -4461,65 +4486,65 @@
       <c r="T45" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V45" s="7" t="e">
-        <f t="shared" ref="V45:AJ45" si="15">_xlfn.RANK.EQ(D45,$D45:$R45,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ45" s="7" t="e">
-        <f t="shared" si="15"/>
-        <v>#N/A</v>
+      <c r="V45" s="7" t="e" cm="1">
+        <f t="array" ref="V45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(D45,2-INT(LOG10(ABS(D45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W45" s="7" t="e" cm="1">
+        <f t="array" ref="W45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(E45,2-INT(LOG10(ABS(E45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X45" s="7" t="e" cm="1">
+        <f t="array" ref="X45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(F45,2-INT(LOG10(ABS(F45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y45" s="7" t="e" cm="1">
+        <f t="array" ref="Y45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(G45,2-INT(LOG10(ABS(G45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z45" s="7" t="e" cm="1">
+        <f t="array" ref="Z45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(H45,2-INT(LOG10(ABS(H45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA45" s="7" t="e" cm="1">
+        <f t="array" ref="AA45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(I45,2-INT(LOG10(ABS(I45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB45" s="7" t="e" cm="1">
+        <f t="array" ref="AB45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(J45,2-INT(LOG10(ABS(J45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC45" s="7" t="e" cm="1">
+        <f t="array" ref="AC45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(K45,2-INT(LOG10(ABS(K45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD45" s="7" t="e" cm="1">
+        <f t="array" ref="AD45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(L45,2-INT(LOG10(ABS(L45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE45" s="7" t="e" cm="1">
+        <f t="array" ref="AE45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(M45,2-INT(LOG10(ABS(M45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF45" s="7" t="e" cm="1">
+        <f t="array" ref="AF45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(N45,2-INT(LOG10(ABS(N45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG45" s="7" t="e" cm="1">
+        <f t="array" ref="AG45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(O45,2-INT(LOG10(ABS(O45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH45" s="7" t="e" cm="1">
+        <f t="array" ref="AH45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(P45,2-INT(LOG10(ABS(P45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI45" s="7" t="e" cm="1">
+        <f t="array" ref="AI45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(Q45,2-INT(LOG10(ABS(Q45))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ45" s="7" t="e" cm="1">
+        <f t="array" ref="AJ45">SUMPRODUCT(--(ROUND($D45:$R45,2-INT(LOG10(ABS($D45:$R45))))&lt;ROUND(R45,2-INT(LOG10(ABS(R45))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="46" spans="1:36" x14ac:dyDescent="0.25">
@@ -4629,65 +4654,65 @@
       <c r="T48" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V48" s="7" t="e">
-        <f t="shared" ref="V48:AJ48" si="16">_xlfn.RANK.EQ(D48,$D48:$R48,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ48" s="7" t="e">
-        <f t="shared" si="16"/>
-        <v>#N/A</v>
+      <c r="V48" s="7" t="e" cm="1">
+        <f t="array" ref="V48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(D48,2-INT(LOG10(ABS(D48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W48" s="7" t="e" cm="1">
+        <f t="array" ref="W48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(E48,2-INT(LOG10(ABS(E48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X48" s="7" t="e" cm="1">
+        <f t="array" ref="X48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(F48,2-INT(LOG10(ABS(F48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y48" s="7" t="e" cm="1">
+        <f t="array" ref="Y48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(G48,2-INT(LOG10(ABS(G48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z48" s="7" t="e" cm="1">
+        <f t="array" ref="Z48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(H48,2-INT(LOG10(ABS(H48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA48" s="7" t="e" cm="1">
+        <f t="array" ref="AA48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(I48,2-INT(LOG10(ABS(I48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB48" s="7" t="e" cm="1">
+        <f t="array" ref="AB48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(J48,2-INT(LOG10(ABS(J48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC48" s="7" t="e" cm="1">
+        <f t="array" ref="AC48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(K48,2-INT(LOG10(ABS(K48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD48" s="7" t="e" cm="1">
+        <f t="array" ref="AD48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(L48,2-INT(LOG10(ABS(L48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE48" s="7" t="e" cm="1">
+        <f t="array" ref="AE48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(M48,2-INT(LOG10(ABS(M48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF48" s="7" t="e" cm="1">
+        <f t="array" ref="AF48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(N48,2-INT(LOG10(ABS(N48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG48" s="7" t="e" cm="1">
+        <f t="array" ref="AG48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(O48,2-INT(LOG10(ABS(O48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH48" s="7" t="e" cm="1">
+        <f t="array" ref="AH48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(P48,2-INT(LOG10(ABS(P48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI48" s="7" t="e" cm="1">
+        <f t="array" ref="AI48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(Q48,2-INT(LOG10(ABS(Q48))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ48" s="7" t="e" cm="1">
+        <f t="array" ref="AJ48">SUMPRODUCT(--(ROUND($D48:$R48,2-INT(LOG10(ABS($D48:$R48))))&lt;ROUND(R48,2-INT(LOG10(ABS(R48))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="49" spans="1:36" x14ac:dyDescent="0.25">
@@ -4799,65 +4824,65 @@
       <c r="T51" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V51" s="7" t="e">
-        <f t="shared" ref="V51:AJ51" si="17">_xlfn.RANK.EQ(D51,$D51:$R51,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ51" s="7" t="e">
-        <f t="shared" si="17"/>
-        <v>#N/A</v>
+      <c r="V51" s="7" t="e" cm="1">
+        <f t="array" ref="V51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(D51,2-INT(LOG10(ABS(D51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W51" s="7" t="e" cm="1">
+        <f t="array" ref="W51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(E51,2-INT(LOG10(ABS(E51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X51" s="7" t="e" cm="1">
+        <f t="array" ref="X51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(F51,2-INT(LOG10(ABS(F51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y51" s="7" t="e" cm="1">
+        <f t="array" ref="Y51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(G51,2-INT(LOG10(ABS(G51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z51" s="7" t="e" cm="1">
+        <f t="array" ref="Z51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(H51,2-INT(LOG10(ABS(H51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA51" s="7" t="e" cm="1">
+        <f t="array" ref="AA51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(I51,2-INT(LOG10(ABS(I51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB51" s="7" t="e" cm="1">
+        <f t="array" ref="AB51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(J51,2-INT(LOG10(ABS(J51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC51" s="7" t="e" cm="1">
+        <f t="array" ref="AC51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(K51,2-INT(LOG10(ABS(K51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD51" s="7" t="e" cm="1">
+        <f t="array" ref="AD51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(L51,2-INT(LOG10(ABS(L51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE51" s="7" t="e" cm="1">
+        <f t="array" ref="AE51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(M51,2-INT(LOG10(ABS(M51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF51" s="7" t="e" cm="1">
+        <f t="array" ref="AF51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(N51,2-INT(LOG10(ABS(N51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG51" s="7" t="e" cm="1">
+        <f t="array" ref="AG51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(O51,2-INT(LOG10(ABS(O51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH51" s="7" t="e" cm="1">
+        <f t="array" ref="AH51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(P51,2-INT(LOG10(ABS(P51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI51" s="7" t="e" cm="1">
+        <f t="array" ref="AI51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(Q51,2-INT(LOG10(ABS(Q51))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ51" s="7" t="e" cm="1">
+        <f t="array" ref="AJ51">SUMPRODUCT(--(ROUND($D51:$R51,2-INT(LOG10(ABS($D51:$R51))))&lt;ROUND(R51,2-INT(LOG10(ABS(R51))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="52" spans="1:36" x14ac:dyDescent="0.25">
@@ -4967,65 +4992,65 @@
       <c r="T54" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V54" s="7" t="e">
-        <f t="shared" ref="V54:AJ54" si="18">_xlfn.RANK.EQ(D54,$D54:$R54,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ54" s="7" t="e">
-        <f t="shared" si="18"/>
-        <v>#N/A</v>
+      <c r="V54" s="7" t="e" cm="1">
+        <f t="array" ref="V54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(D54,2-INT(LOG10(ABS(D54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W54" s="7" t="e" cm="1">
+        <f t="array" ref="W54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(E54,2-INT(LOG10(ABS(E54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X54" s="7" t="e" cm="1">
+        <f t="array" ref="X54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(F54,2-INT(LOG10(ABS(F54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y54" s="7" t="e" cm="1">
+        <f t="array" ref="Y54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(G54,2-INT(LOG10(ABS(G54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z54" s="7" t="e" cm="1">
+        <f t="array" ref="Z54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(H54,2-INT(LOG10(ABS(H54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA54" s="7" t="e" cm="1">
+        <f t="array" ref="AA54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(I54,2-INT(LOG10(ABS(I54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB54" s="7" t="e" cm="1">
+        <f t="array" ref="AB54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(J54,2-INT(LOG10(ABS(J54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC54" s="7" t="e" cm="1">
+        <f t="array" ref="AC54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(K54,2-INT(LOG10(ABS(K54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD54" s="7" t="e" cm="1">
+        <f t="array" ref="AD54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(L54,2-INT(LOG10(ABS(L54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE54" s="7" t="e" cm="1">
+        <f t="array" ref="AE54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(M54,2-INT(LOG10(ABS(M54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF54" s="7" t="e" cm="1">
+        <f t="array" ref="AF54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(N54,2-INT(LOG10(ABS(N54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG54" s="7" t="e" cm="1">
+        <f t="array" ref="AG54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(O54,2-INT(LOG10(ABS(O54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH54" s="7" t="e" cm="1">
+        <f t="array" ref="AH54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(P54,2-INT(LOG10(ABS(P54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI54" s="7" t="e" cm="1">
+        <f t="array" ref="AI54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(Q54,2-INT(LOG10(ABS(Q54))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ54" s="7" t="e" cm="1">
+        <f t="array" ref="AJ54">SUMPRODUCT(--(ROUND($D54:$R54,2-INT(LOG10(ABS($D54:$R54))))&lt;ROUND(R54,2-INT(LOG10(ABS(R54))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="55" spans="1:36" x14ac:dyDescent="0.25">
@@ -5135,65 +5160,65 @@
       <c r="T57" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V57" s="7" t="e">
-        <f t="shared" ref="V57:AJ57" si="19">_xlfn.RANK.EQ(D57,$D57:$R57,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ57" s="7" t="e">
-        <f t="shared" si="19"/>
-        <v>#N/A</v>
+      <c r="V57" s="7" t="e" cm="1">
+        <f t="array" ref="V57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(D57,2-INT(LOG10(ABS(D57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W57" s="7" t="e" cm="1">
+        <f t="array" ref="W57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(E57,2-INT(LOG10(ABS(E57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X57" s="7" t="e" cm="1">
+        <f t="array" ref="X57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(F57,2-INT(LOG10(ABS(F57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y57" s="7" t="e" cm="1">
+        <f t="array" ref="Y57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(G57,2-INT(LOG10(ABS(G57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z57" s="7" t="e" cm="1">
+        <f t="array" ref="Z57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(H57,2-INT(LOG10(ABS(H57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA57" s="7" t="e" cm="1">
+        <f t="array" ref="AA57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(I57,2-INT(LOG10(ABS(I57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB57" s="7" t="e" cm="1">
+        <f t="array" ref="AB57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(J57,2-INT(LOG10(ABS(J57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC57" s="7" t="e" cm="1">
+        <f t="array" ref="AC57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(K57,2-INT(LOG10(ABS(K57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD57" s="7" t="e" cm="1">
+        <f t="array" ref="AD57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(L57,2-INT(LOG10(ABS(L57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE57" s="7" t="e" cm="1">
+        <f t="array" ref="AE57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(M57,2-INT(LOG10(ABS(M57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF57" s="7" t="e" cm="1">
+        <f t="array" ref="AF57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(N57,2-INT(LOG10(ABS(N57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG57" s="7" t="e" cm="1">
+        <f t="array" ref="AG57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(O57,2-INT(LOG10(ABS(O57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH57" s="7" t="e" cm="1">
+        <f t="array" ref="AH57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(P57,2-INT(LOG10(ABS(P57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI57" s="7" t="e" cm="1">
+        <f t="array" ref="AI57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(Q57,2-INT(LOG10(ABS(Q57))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ57" s="7" t="e" cm="1">
+        <f t="array" ref="AJ57">SUMPRODUCT(--(ROUND($D57:$R57,2-INT(LOG10(ABS($D57:$R57))))&lt;ROUND(R57,2-INT(LOG10(ABS(R57))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="58" spans="1:36" x14ac:dyDescent="0.25">
@@ -5303,65 +5328,65 @@
       <c r="T60" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V60" s="7" t="e">
-        <f t="shared" ref="V60:AJ60" si="20">_xlfn.RANK.EQ(D60,$D60:$R60,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ60" s="7" t="e">
-        <f t="shared" si="20"/>
-        <v>#N/A</v>
+      <c r="V60" s="7" t="e" cm="1">
+        <f t="array" ref="V60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(D60,2-INT(LOG10(ABS(D60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W60" s="7" t="e" cm="1">
+        <f t="array" ref="W60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(E60,2-INT(LOG10(ABS(E60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X60" s="7" t="e" cm="1">
+        <f t="array" ref="X60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(F60,2-INT(LOG10(ABS(F60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y60" s="7" t="e" cm="1">
+        <f t="array" ref="Y60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(G60,2-INT(LOG10(ABS(G60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z60" s="7" t="e" cm="1">
+        <f t="array" ref="Z60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(H60,2-INT(LOG10(ABS(H60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA60" s="7" t="e" cm="1">
+        <f t="array" ref="AA60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(I60,2-INT(LOG10(ABS(I60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB60" s="7" t="e" cm="1">
+        <f t="array" ref="AB60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(J60,2-INT(LOG10(ABS(J60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC60" s="7" t="e" cm="1">
+        <f t="array" ref="AC60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(K60,2-INT(LOG10(ABS(K60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD60" s="7" t="e" cm="1">
+        <f t="array" ref="AD60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(L60,2-INT(LOG10(ABS(L60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE60" s="7" t="e" cm="1">
+        <f t="array" ref="AE60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(M60,2-INT(LOG10(ABS(M60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF60" s="7" t="e" cm="1">
+        <f t="array" ref="AF60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(N60,2-INT(LOG10(ABS(N60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG60" s="7" t="e" cm="1">
+        <f t="array" ref="AG60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(O60,2-INT(LOG10(ABS(O60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH60" s="7" t="e" cm="1">
+        <f t="array" ref="AH60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(P60,2-INT(LOG10(ABS(P60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI60" s="7" t="e" cm="1">
+        <f t="array" ref="AI60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(Q60,2-INT(LOG10(ABS(Q60))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ60" s="7" t="e" cm="1">
+        <f t="array" ref="AJ60">SUMPRODUCT(--(ROUND($D60:$R60,2-INT(LOG10(ABS($D60:$R60))))&lt;ROUND(R60,2-INT(LOG10(ABS(R60))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="61" spans="1:36" x14ac:dyDescent="0.25">
@@ -5471,65 +5496,65 @@
       <c r="T63" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V63" s="7" t="e">
-        <f t="shared" ref="V63:AJ63" si="21">_xlfn.RANK.EQ(D63,$D63:$R63,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ63" s="7" t="e">
-        <f t="shared" si="21"/>
-        <v>#N/A</v>
+      <c r="V63" s="7" t="e" cm="1">
+        <f t="array" ref="V63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(D63,2-INT(LOG10(ABS(D63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W63" s="7" t="e" cm="1">
+        <f t="array" ref="W63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(E63,2-INT(LOG10(ABS(E63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X63" s="7" t="e" cm="1">
+        <f t="array" ref="X63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(F63,2-INT(LOG10(ABS(F63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y63" s="7" t="e" cm="1">
+        <f t="array" ref="Y63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(G63,2-INT(LOG10(ABS(G63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z63" s="7" t="e" cm="1">
+        <f t="array" ref="Z63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(H63,2-INT(LOG10(ABS(H63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA63" s="7" t="e" cm="1">
+        <f t="array" ref="AA63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(I63,2-INT(LOG10(ABS(I63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB63" s="7" t="e" cm="1">
+        <f t="array" ref="AB63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(J63,2-INT(LOG10(ABS(J63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC63" s="7" t="e" cm="1">
+        <f t="array" ref="AC63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(K63,2-INT(LOG10(ABS(K63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD63" s="7" t="e" cm="1">
+        <f t="array" ref="AD63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(L63,2-INT(LOG10(ABS(L63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE63" s="7" t="e" cm="1">
+        <f t="array" ref="AE63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(M63,2-INT(LOG10(ABS(M63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF63" s="7" t="e" cm="1">
+        <f t="array" ref="AF63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(N63,2-INT(LOG10(ABS(N63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG63" s="7" t="e" cm="1">
+        <f t="array" ref="AG63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(O63,2-INT(LOG10(ABS(O63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH63" s="7" t="e" cm="1">
+        <f t="array" ref="AH63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(P63,2-INT(LOG10(ABS(P63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI63" s="7" t="e" cm="1">
+        <f t="array" ref="AI63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(Q63,2-INT(LOG10(ABS(Q63))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ63" s="7" t="e" cm="1">
+        <f t="array" ref="AJ63">SUMPRODUCT(--(ROUND($D63:$R63,2-INT(LOG10(ABS($D63:$R63))))&lt;ROUND(R63,2-INT(LOG10(ABS(R63))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="64" spans="1:36" x14ac:dyDescent="0.25">
@@ -5639,65 +5664,65 @@
       <c r="T66" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V66" s="7" t="e">
-        <f t="shared" ref="V66:AJ66" si="22">_xlfn.RANK.EQ(D66,$D66:$R66,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ66" s="7" t="e">
-        <f t="shared" si="22"/>
-        <v>#N/A</v>
+      <c r="V66" s="7" t="e" cm="1">
+        <f t="array" ref="V66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(D66,2-INT(LOG10(ABS(D66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W66" s="7" t="e" cm="1">
+        <f t="array" ref="W66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(E66,2-INT(LOG10(ABS(E66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X66" s="7" t="e" cm="1">
+        <f t="array" ref="X66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(F66,2-INT(LOG10(ABS(F66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y66" s="7" t="e" cm="1">
+        <f t="array" ref="Y66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(G66,2-INT(LOG10(ABS(G66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z66" s="7" t="e" cm="1">
+        <f t="array" ref="Z66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(H66,2-INT(LOG10(ABS(H66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA66" s="7" t="e" cm="1">
+        <f t="array" ref="AA66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(I66,2-INT(LOG10(ABS(I66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB66" s="7" t="e" cm="1">
+        <f t="array" ref="AB66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(J66,2-INT(LOG10(ABS(J66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC66" s="7" t="e" cm="1">
+        <f t="array" ref="AC66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(K66,2-INT(LOG10(ABS(K66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD66" s="7" t="e" cm="1">
+        <f t="array" ref="AD66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(L66,2-INT(LOG10(ABS(L66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE66" s="7" t="e" cm="1">
+        <f t="array" ref="AE66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(M66,2-INT(LOG10(ABS(M66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF66" s="7" t="e" cm="1">
+        <f t="array" ref="AF66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(N66,2-INT(LOG10(ABS(N66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG66" s="7" t="e" cm="1">
+        <f t="array" ref="AG66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(O66,2-INT(LOG10(ABS(O66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH66" s="7" t="e" cm="1">
+        <f t="array" ref="AH66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(P66,2-INT(LOG10(ABS(P66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI66" s="7" t="e" cm="1">
+        <f t="array" ref="AI66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(Q66,2-INT(LOG10(ABS(Q66))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ66" s="7" t="e" cm="1">
+        <f t="array" ref="AJ66">SUMPRODUCT(--(ROUND($D66:$R66,2-INT(LOG10(ABS($D66:$R66))))&lt;ROUND(R66,2-INT(LOG10(ABS(R66))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="67" spans="1:36" x14ac:dyDescent="0.25">
@@ -5809,65 +5834,65 @@
       <c r="T69" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V69" s="7" t="e">
-        <f t="shared" ref="V69:AJ69" si="23">_xlfn.RANK.EQ(D69,$D69:$R69,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ69" s="7" t="e">
-        <f t="shared" si="23"/>
-        <v>#N/A</v>
+      <c r="V69" s="7" t="e" cm="1">
+        <f t="array" ref="V69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(D69,2-INT(LOG10(ABS(D69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W69" s="7" t="e" cm="1">
+        <f t="array" ref="W69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(E69,2-INT(LOG10(ABS(E69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X69" s="7" t="e" cm="1">
+        <f t="array" ref="X69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(F69,2-INT(LOG10(ABS(F69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y69" s="7" t="e" cm="1">
+        <f t="array" ref="Y69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(G69,2-INT(LOG10(ABS(G69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z69" s="7" t="e" cm="1">
+        <f t="array" ref="Z69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(H69,2-INT(LOG10(ABS(H69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA69" s="7" t="e" cm="1">
+        <f t="array" ref="AA69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(I69,2-INT(LOG10(ABS(I69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB69" s="7" t="e" cm="1">
+        <f t="array" ref="AB69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(J69,2-INT(LOG10(ABS(J69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC69" s="7" t="e" cm="1">
+        <f t="array" ref="AC69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(K69,2-INT(LOG10(ABS(K69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD69" s="7" t="e" cm="1">
+        <f t="array" ref="AD69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(L69,2-INT(LOG10(ABS(L69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE69" s="7" t="e" cm="1">
+        <f t="array" ref="AE69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(M69,2-INT(LOG10(ABS(M69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF69" s="7" t="e" cm="1">
+        <f t="array" ref="AF69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(N69,2-INT(LOG10(ABS(N69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG69" s="7" t="e" cm="1">
+        <f t="array" ref="AG69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(O69,2-INT(LOG10(ABS(O69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH69" s="7" t="e" cm="1">
+        <f t="array" ref="AH69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(P69,2-INT(LOG10(ABS(P69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI69" s="7" t="e" cm="1">
+        <f t="array" ref="AI69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(Q69,2-INT(LOG10(ABS(Q69))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ69" s="7" t="e" cm="1">
+        <f t="array" ref="AJ69">SUMPRODUCT(--(ROUND($D69:$R69,2-INT(LOG10(ABS($D69:$R69))))&lt;ROUND(R69,2-INT(LOG10(ABS(R69))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="70" spans="1:36" x14ac:dyDescent="0.25">
@@ -5977,65 +6002,65 @@
       <c r="T72" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V72" s="7" t="e">
-        <f t="shared" ref="V72:AJ72" si="24">_xlfn.RANK.EQ(D72,$D72:$R72,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ72" s="7" t="e">
-        <f t="shared" si="24"/>
-        <v>#N/A</v>
+      <c r="V72" s="7" t="e" cm="1">
+        <f t="array" ref="V72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(D72,2-INT(LOG10(ABS(D72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W72" s="7" t="e" cm="1">
+        <f t="array" ref="W72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(E72,2-INT(LOG10(ABS(E72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X72" s="7" t="e" cm="1">
+        <f t="array" ref="X72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(F72,2-INT(LOG10(ABS(F72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y72" s="7" t="e" cm="1">
+        <f t="array" ref="Y72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(G72,2-INT(LOG10(ABS(G72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z72" s="7" t="e" cm="1">
+        <f t="array" ref="Z72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(H72,2-INT(LOG10(ABS(H72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA72" s="7" t="e" cm="1">
+        <f t="array" ref="AA72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(I72,2-INT(LOG10(ABS(I72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB72" s="7" t="e" cm="1">
+        <f t="array" ref="AB72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(J72,2-INT(LOG10(ABS(J72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC72" s="7" t="e" cm="1">
+        <f t="array" ref="AC72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(K72,2-INT(LOG10(ABS(K72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD72" s="7" t="e" cm="1">
+        <f t="array" ref="AD72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(L72,2-INT(LOG10(ABS(L72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE72" s="7" t="e" cm="1">
+        <f t="array" ref="AE72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(M72,2-INT(LOG10(ABS(M72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF72" s="7" t="e" cm="1">
+        <f t="array" ref="AF72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(N72,2-INT(LOG10(ABS(N72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG72" s="7" t="e" cm="1">
+        <f t="array" ref="AG72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(O72,2-INT(LOG10(ABS(O72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH72" s="7" t="e" cm="1">
+        <f t="array" ref="AH72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(P72,2-INT(LOG10(ABS(P72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI72" s="7" t="e" cm="1">
+        <f t="array" ref="AI72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(Q72,2-INT(LOG10(ABS(Q72))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ72" s="7" t="e" cm="1">
+        <f t="array" ref="AJ72">SUMPRODUCT(--(ROUND($D72:$R72,2-INT(LOG10(ABS($D72:$R72))))&lt;ROUND(R72,2-INT(LOG10(ABS(R72))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="73" spans="1:36" x14ac:dyDescent="0.25">
@@ -6145,65 +6170,65 @@
       <c r="T75" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V75" s="7" t="e">
-        <f t="shared" ref="V75:AJ75" si="25">_xlfn.RANK.EQ(D75,$D75:$R75,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ75" s="7" t="e">
-        <f t="shared" si="25"/>
-        <v>#N/A</v>
+      <c r="V75" s="7" t="e" cm="1">
+        <f t="array" ref="V75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(D75,2-INT(LOG10(ABS(D75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W75" s="7" t="e" cm="1">
+        <f t="array" ref="W75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(E75,2-INT(LOG10(ABS(E75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X75" s="7" t="e" cm="1">
+        <f t="array" ref="X75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(F75,2-INT(LOG10(ABS(F75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y75" s="7" t="e" cm="1">
+        <f t="array" ref="Y75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(G75,2-INT(LOG10(ABS(G75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z75" s="7" t="e" cm="1">
+        <f t="array" ref="Z75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(H75,2-INT(LOG10(ABS(H75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA75" s="7" t="e" cm="1">
+        <f t="array" ref="AA75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(I75,2-INT(LOG10(ABS(I75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB75" s="7" t="e" cm="1">
+        <f t="array" ref="AB75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(J75,2-INT(LOG10(ABS(J75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC75" s="7" t="e" cm="1">
+        <f t="array" ref="AC75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(K75,2-INT(LOG10(ABS(K75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD75" s="7" t="e" cm="1">
+        <f t="array" ref="AD75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(L75,2-INT(LOG10(ABS(L75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE75" s="7" t="e" cm="1">
+        <f t="array" ref="AE75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(M75,2-INT(LOG10(ABS(M75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF75" s="7" t="e" cm="1">
+        <f t="array" ref="AF75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(N75,2-INT(LOG10(ABS(N75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG75" s="7" t="e" cm="1">
+        <f t="array" ref="AG75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(O75,2-INT(LOG10(ABS(O75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH75" s="7" t="e" cm="1">
+        <f t="array" ref="AH75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(P75,2-INT(LOG10(ABS(P75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI75" s="7" t="e" cm="1">
+        <f t="array" ref="AI75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(Q75,2-INT(LOG10(ABS(Q75))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ75" s="7" t="e" cm="1">
+        <f t="array" ref="AJ75">SUMPRODUCT(--(ROUND($D75:$R75,2-INT(LOG10(ABS($D75:$R75))))&lt;ROUND(R75,2-INT(LOG10(ABS(R75))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="76" spans="1:36" x14ac:dyDescent="0.25">
@@ -6313,65 +6338,65 @@
       <c r="T78" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V78" s="7" t="e">
-        <f t="shared" ref="V78:AJ78" si="26">_xlfn.RANK.EQ(D78,$D78:$R78,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ78" s="7" t="e">
-        <f t="shared" si="26"/>
-        <v>#N/A</v>
+      <c r="V78" s="7" t="e" cm="1">
+        <f t="array" ref="V78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(D78,2-INT(LOG10(ABS(D78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W78" s="7" t="e" cm="1">
+        <f t="array" ref="W78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(E78,2-INT(LOG10(ABS(E78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X78" s="7" t="e" cm="1">
+        <f t="array" ref="X78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(F78,2-INT(LOG10(ABS(F78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y78" s="7" t="e" cm="1">
+        <f t="array" ref="Y78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(G78,2-INT(LOG10(ABS(G78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z78" s="7" t="e" cm="1">
+        <f t="array" ref="Z78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(H78,2-INT(LOG10(ABS(H78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA78" s="7" t="e" cm="1">
+        <f t="array" ref="AA78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(I78,2-INT(LOG10(ABS(I78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB78" s="7" t="e" cm="1">
+        <f t="array" ref="AB78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(J78,2-INT(LOG10(ABS(J78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC78" s="7" t="e" cm="1">
+        <f t="array" ref="AC78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(K78,2-INT(LOG10(ABS(K78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD78" s="7" t="e" cm="1">
+        <f t="array" ref="AD78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(L78,2-INT(LOG10(ABS(L78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE78" s="7" t="e" cm="1">
+        <f t="array" ref="AE78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(M78,2-INT(LOG10(ABS(M78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF78" s="7" t="e" cm="1">
+        <f t="array" ref="AF78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(N78,2-INT(LOG10(ABS(N78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG78" s="7" t="e" cm="1">
+        <f t="array" ref="AG78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(O78,2-INT(LOG10(ABS(O78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH78" s="7" t="e" cm="1">
+        <f t="array" ref="AH78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(P78,2-INT(LOG10(ABS(P78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI78" s="7" t="e" cm="1">
+        <f t="array" ref="AI78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(Q78,2-INT(LOG10(ABS(Q78))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ78" s="7" t="e" cm="1">
+        <f t="array" ref="AJ78">SUMPRODUCT(--(ROUND($D78:$R78,2-INT(LOG10(ABS($D78:$R78))))&lt;ROUND(R78,2-INT(LOG10(ABS(R78))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="79" spans="1:36" x14ac:dyDescent="0.25">
@@ -6481,65 +6506,65 @@
       <c r="T81" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V81" s="7" t="e">
-        <f t="shared" ref="V81:AJ81" si="27">_xlfn.RANK.EQ(D81,$D81:$R81,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ81" s="7" t="e">
-        <f t="shared" si="27"/>
-        <v>#N/A</v>
+      <c r="V81" s="7" t="e" cm="1">
+        <f t="array" ref="V81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(D81,2-INT(LOG10(ABS(D81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W81" s="7" t="e" cm="1">
+        <f t="array" ref="W81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(E81,2-INT(LOG10(ABS(E81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X81" s="7" t="e" cm="1">
+        <f t="array" ref="X81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(F81,2-INT(LOG10(ABS(F81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y81" s="7" t="e" cm="1">
+        <f t="array" ref="Y81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(G81,2-INT(LOG10(ABS(G81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z81" s="7" t="e" cm="1">
+        <f t="array" ref="Z81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(H81,2-INT(LOG10(ABS(H81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA81" s="7" t="e" cm="1">
+        <f t="array" ref="AA81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(I81,2-INT(LOG10(ABS(I81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB81" s="7" t="e" cm="1">
+        <f t="array" ref="AB81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(J81,2-INT(LOG10(ABS(J81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC81" s="7" t="e" cm="1">
+        <f t="array" ref="AC81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(K81,2-INT(LOG10(ABS(K81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD81" s="7" t="e" cm="1">
+        <f t="array" ref="AD81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(L81,2-INT(LOG10(ABS(L81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE81" s="7" t="e" cm="1">
+        <f t="array" ref="AE81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(M81,2-INT(LOG10(ABS(M81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF81" s="7" t="e" cm="1">
+        <f t="array" ref="AF81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(N81,2-INT(LOG10(ABS(N81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG81" s="7" t="e" cm="1">
+        <f t="array" ref="AG81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(O81,2-INT(LOG10(ABS(O81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH81" s="7" t="e" cm="1">
+        <f t="array" ref="AH81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(P81,2-INT(LOG10(ABS(P81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI81" s="7" t="e" cm="1">
+        <f t="array" ref="AI81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(Q81,2-INT(LOG10(ABS(Q81))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ81" s="7" t="e" cm="1">
+        <f t="array" ref="AJ81">SUMPRODUCT(--(ROUND($D81:$R81,2-INT(LOG10(ABS($D81:$R81))))&lt;ROUND(R81,2-INT(LOG10(ABS(R81))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="82" spans="1:36" x14ac:dyDescent="0.25">
@@ -6649,65 +6674,65 @@
       <c r="T84" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V84" s="7" t="e">
-        <f t="shared" ref="V84:AJ84" si="28">_xlfn.RANK.EQ(D84,$D84:$R84,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ84" s="7" t="e">
-        <f t="shared" si="28"/>
-        <v>#N/A</v>
+      <c r="V84" s="7" t="e" cm="1">
+        <f t="array" ref="V84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(D84,2-INT(LOG10(ABS(D84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W84" s="7" t="e" cm="1">
+        <f t="array" ref="W84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(E84,2-INT(LOG10(ABS(E84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X84" s="7" t="e" cm="1">
+        <f t="array" ref="X84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(F84,2-INT(LOG10(ABS(F84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y84" s="7" t="e" cm="1">
+        <f t="array" ref="Y84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(G84,2-INT(LOG10(ABS(G84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z84" s="7" t="e" cm="1">
+        <f t="array" ref="Z84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(H84,2-INT(LOG10(ABS(H84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA84" s="7" t="e" cm="1">
+        <f t="array" ref="AA84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(I84,2-INT(LOG10(ABS(I84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB84" s="7" t="e" cm="1">
+        <f t="array" ref="AB84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(J84,2-INT(LOG10(ABS(J84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC84" s="7" t="e" cm="1">
+        <f t="array" ref="AC84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(K84,2-INT(LOG10(ABS(K84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD84" s="7" t="e" cm="1">
+        <f t="array" ref="AD84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(L84,2-INT(LOG10(ABS(L84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE84" s="7" t="e" cm="1">
+        <f t="array" ref="AE84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(M84,2-INT(LOG10(ABS(M84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF84" s="7" t="e" cm="1">
+        <f t="array" ref="AF84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(N84,2-INT(LOG10(ABS(N84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG84" s="7" t="e" cm="1">
+        <f t="array" ref="AG84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(O84,2-INT(LOG10(ABS(O84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH84" s="7" t="e" cm="1">
+        <f t="array" ref="AH84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(P84,2-INT(LOG10(ABS(P84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI84" s="7" t="e" cm="1">
+        <f t="array" ref="AI84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(Q84,2-INT(LOG10(ABS(Q84))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ84" s="7" t="e" cm="1">
+        <f t="array" ref="AJ84">SUMPRODUCT(--(ROUND($D84:$R84,2-INT(LOG10(ABS($D84:$R84))))&lt;ROUND(R84,2-INT(LOG10(ABS(R84))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="85" spans="1:36" x14ac:dyDescent="0.25">
@@ -6817,65 +6842,65 @@
       <c r="T87" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V87" s="7" t="e">
-        <f t="shared" ref="V87:AJ87" si="29">_xlfn.RANK.EQ(D87,$D87:$R87,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ87" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
+      <c r="V87" s="7" t="e" cm="1">
+        <f t="array" ref="V87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(D87,2-INT(LOG10(ABS(D87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W87" s="7" t="e" cm="1">
+        <f t="array" ref="W87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(E87,2-INT(LOG10(ABS(E87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X87" s="7" t="e" cm="1">
+        <f t="array" ref="X87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(F87,2-INT(LOG10(ABS(F87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y87" s="7" t="e" cm="1">
+        <f t="array" ref="Y87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(G87,2-INT(LOG10(ABS(G87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z87" s="7" t="e" cm="1">
+        <f t="array" ref="Z87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(H87,2-INT(LOG10(ABS(H87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA87" s="7" t="e" cm="1">
+        <f t="array" ref="AA87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(I87,2-INT(LOG10(ABS(I87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB87" s="7" t="e" cm="1">
+        <f t="array" ref="AB87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(J87,2-INT(LOG10(ABS(J87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC87" s="7" t="e" cm="1">
+        <f t="array" ref="AC87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(K87,2-INT(LOG10(ABS(K87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD87" s="7" t="e" cm="1">
+        <f t="array" ref="AD87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(L87,2-INT(LOG10(ABS(L87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE87" s="7" t="e" cm="1">
+        <f t="array" ref="AE87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(M87,2-INT(LOG10(ABS(M87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF87" s="7" t="e" cm="1">
+        <f t="array" ref="AF87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(N87,2-INT(LOG10(ABS(N87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG87" s="7" t="e" cm="1">
+        <f t="array" ref="AG87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(O87,2-INT(LOG10(ABS(O87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH87" s="7" t="e" cm="1">
+        <f t="array" ref="AH87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(P87,2-INT(LOG10(ABS(P87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI87" s="7" t="e" cm="1">
+        <f t="array" ref="AI87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(Q87,2-INT(LOG10(ABS(Q87))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ87" s="7" t="e" cm="1">
+        <f t="array" ref="AJ87">SUMPRODUCT(--(ROUND($D87:$R87,2-INT(LOG10(ABS($D87:$R87))))&lt;ROUND(R87,2-INT(LOG10(ABS(R87))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="88" spans="1:36" x14ac:dyDescent="0.25">
@@ -6985,65 +7010,65 @@
       <c r="T90" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V90" s="7" t="e">
-        <f t="shared" ref="V90:AJ90" si="30">_xlfn.RANK.EQ(D90,$D90:$R90,1)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="X90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Y90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="Z90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AA90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AB90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AC90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AD90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AE90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AF90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AG90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AH90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AI90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="AJ90" s="7" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
+      <c r="V90" s="7" t="e" cm="1">
+        <f t="array" ref="V90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(D90,2-INT(LOG10(ABS(D90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="W90" s="7" t="e" cm="1">
+        <f t="array" ref="W90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(E90,2-INT(LOG10(ABS(E90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="X90" s="7" t="e" cm="1">
+        <f t="array" ref="X90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(F90,2-INT(LOG10(ABS(F90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Y90" s="7" t="e" cm="1">
+        <f t="array" ref="Y90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(G90,2-INT(LOG10(ABS(G90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="Z90" s="7" t="e" cm="1">
+        <f t="array" ref="Z90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(H90,2-INT(LOG10(ABS(H90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AA90" s="7" t="e" cm="1">
+        <f t="array" ref="AA90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(I90,2-INT(LOG10(ABS(I90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AB90" s="7" t="e" cm="1">
+        <f t="array" ref="AB90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(J90,2-INT(LOG10(ABS(J90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AC90" s="7" t="e" cm="1">
+        <f t="array" ref="AC90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(K90,2-INT(LOG10(ABS(K90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AD90" s="7" t="e" cm="1">
+        <f t="array" ref="AD90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(L90,2-INT(LOG10(ABS(L90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AE90" s="7" t="e" cm="1">
+        <f t="array" ref="AE90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(M90,2-INT(LOG10(ABS(M90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AF90" s="7" t="e" cm="1">
+        <f t="array" ref="AF90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(N90,2-INT(LOG10(ABS(N90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AG90" s="7" t="e" cm="1">
+        <f t="array" ref="AG90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(O90,2-INT(LOG10(ABS(O90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AH90" s="7" t="e" cm="1">
+        <f t="array" ref="AH90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(P90,2-INT(LOG10(ABS(P90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AI90" s="7" t="e" cm="1">
+        <f t="array" ref="AI90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(Q90,2-INT(LOG10(ABS(Q90))))))+1</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AJ90" s="7" t="e" cm="1">
+        <f t="array" ref="AJ90">SUMPRODUCT(--(ROUND($D90:$R90,2-INT(LOG10(ABS($D90:$R90))))&lt;ROUND(R90,2-INT(LOG10(ABS(R90))))))+1</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="91" spans="1:36" x14ac:dyDescent="0.25">
@@ -7135,59 +7160,59 @@
         <v>0</v>
       </c>
       <c r="E93" s="2">
-        <f t="shared" ref="E93:R93" si="31">COUNTIF(W3:W92,1)</f>
+        <f t="shared" ref="E93:R93" si="1">COUNTIF(W3:W92,1)</f>
         <v>0</v>
       </c>
       <c r="F93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R93" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -7202,59 +7227,59 @@
         <v>1</v>
       </c>
       <c r="E94" s="9">
-        <f t="shared" ref="E94:R94" si="32">_xlfn.RANK.EQ(E93,$D93:$R93,0)</f>
+        <f t="shared" ref="E94:R94" si="2">_xlfn.RANK.EQ(E93,$D93:$R93,0)</f>
         <v>1</v>
       </c>
       <c r="F94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="G94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="H94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="I94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="J94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="K94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="L94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="M94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="N94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="O94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="P94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="R94" s="9">
-        <f t="shared" si="32"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -7266,63 +7291,63 @@
       <c r="C95" s="22"/>
       <c r="D95" s="15" t="e">
         <f>AVERAGE(V3:V92)</f>
-        <v>#N/A</v>
+        <v>#NUM!</v>
       </c>
       <c r="E95" s="15" t="e">
-        <f t="shared" ref="E95:R95" si="33">AVERAGE(W3:W92)</f>
-        <v>#N/A</v>
+        <f t="shared" ref="E95:R95" si="3">AVERAGE(W3:W92)</f>
+        <v>#NUM!</v>
       </c>
       <c r="F95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="G95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="H95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="I95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="J95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="K95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="L95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="M95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="N95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="O95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="P95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="Q95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
       <c r="R95" s="15" t="e">
-        <f t="shared" si="33"/>
-        <v>#N/A</v>
+        <f t="shared" si="3"/>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="96" spans="1:36" s="7" customFormat="1" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -7333,63 +7358,63 @@
       <c r="C96" s="25"/>
       <c r="D96" s="5" t="e">
         <f>_xlfn.RANK.EQ(D95,$D95:$R95,1)</f>
-        <v>#N/A</v>
+        <v>#NUM!</v>
       </c>
       <c r="E96" s="5" t="e">
-        <f t="shared" ref="E96:R96" si="34">_xlfn.RANK.EQ(E95,$D95:$R95,1)</f>
-        <v>#N/A</v>
+        <f t="shared" ref="E96:R96" si="4">_xlfn.RANK.EQ(E95,$D95:$R95,1)</f>
+        <v>#NUM!</v>
       </c>
       <c r="F96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="G96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="H96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="I96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="J96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="K96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="L96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="M96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="N96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="O96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="P96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="Q96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
       <c r="R96" s="5" t="e">
-        <f t="shared" si="34"/>
-        <v>#N/A</v>
+        <f t="shared" si="4"/>
+        <v>#NUM!</v>
       </c>
     </row>
   </sheetData>
@@ -7406,94 +7431,154 @@
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="D3:R3">
-    <cfRule type="top10" dxfId="33" priority="30" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="33" priority="30">
+      <formula>ROUND(D3,2-INT(LOG10(ABS(D3))))= ROUND(MIN($D3:$R3),2-INT(LOG10(ABS(MIN($D3:$R3)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:R6">
-    <cfRule type="top10" dxfId="32" priority="29" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="32" priority="29">
+      <formula>ROUND(D6,2-INT(LOG10(ABS(D6))))= ROUND(MIN($D6:$R6),2-INT(LOG10(ABS(MIN($D6:$R6)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:R9">
-    <cfRule type="top10" dxfId="31" priority="28" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="31" priority="28">
+      <formula>ROUND(D9,2-INT(LOG10(ABS(D9))))= ROUND(MIN($D9:$R9),2-INT(LOG10(ABS(MIN($D9:$R9)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D12:R12">
-    <cfRule type="top10" dxfId="30" priority="27" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="30" priority="27">
+      <formula>ROUND(D12,2-INT(LOG10(ABS(D12))))= ROUND(MIN($D12:$R12),2-INT(LOG10(ABS(MIN($D12:$R12)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15:R15">
-    <cfRule type="top10" dxfId="29" priority="26" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="29" priority="26">
+      <formula>ROUND(D15,2-INT(LOG10(ABS(D15))))= ROUND(MIN($D15:$R15),2-INT(LOG10(ABS(MIN($D15:$R15)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:R18">
-    <cfRule type="top10" dxfId="28" priority="25" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="28" priority="25">
+      <formula>ROUND(D18,2-INT(LOG10(ABS(D18))))= ROUND(MIN($D18:$R18),2-INT(LOG10(ABS(MIN($D18:$R18)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D21:R21">
-    <cfRule type="top10" dxfId="27" priority="24" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="27" priority="24">
+      <formula>ROUND(D21,2-INT(LOG10(ABS(D21))))= ROUND(MIN($D21:$R21),2-INT(LOG10(ABS(MIN($D21:$R21)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D24:R24">
-    <cfRule type="top10" dxfId="26" priority="23" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="26" priority="23">
+      <formula>ROUND(D24,2-INT(LOG10(ABS(D24))))= ROUND(MIN($D24:$R24),2-INT(LOG10(ABS(MIN($D24:$R24)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D27:R27">
-    <cfRule type="top10" dxfId="25" priority="22" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="25" priority="22">
+      <formula>ROUND(D27,2-INT(LOG10(ABS(D27))))= ROUND(MIN($D27:$R27),2-INT(LOG10(ABS(MIN($D27:$R27)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D30:R30">
-    <cfRule type="top10" dxfId="24" priority="21" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="24" priority="21">
+      <formula>ROUND(D30,2-INT(LOG10(ABS(D30))))= ROUND(MIN($D30:$R30),2-INT(LOG10(ABS(MIN($D30:$R30)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D33:R33">
-    <cfRule type="top10" dxfId="23" priority="20" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="23" priority="20">
+      <formula>ROUND(D33,2-INT(LOG10(ABS(D33))))= ROUND(MIN($D33:$R33),2-INT(LOG10(ABS(MIN($D33:$R33)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D36:R36">
-    <cfRule type="top10" dxfId="22" priority="19" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="22" priority="19">
+      <formula>ROUND(D36,2-INT(LOG10(ABS(D36))))= ROUND(MIN($D36:$R36),2-INT(LOG10(ABS(MIN($D36:$R36)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D39:R39">
-    <cfRule type="top10" dxfId="21" priority="18" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="21" priority="18">
+      <formula>ROUND(D39,2-INT(LOG10(ABS(D39))))= ROUND(MIN($D39:$R39),2-INT(LOG10(ABS(MIN($D39:$R39)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D42:R42">
-    <cfRule type="top10" dxfId="20" priority="17" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="20" priority="17">
+      <formula>ROUND(D42,2-INT(LOG10(ABS(D42))))= ROUND(MIN($D42:$R42),2-INT(LOG10(ABS(MIN($D42:$R42)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D45:R45">
-    <cfRule type="top10" dxfId="19" priority="16" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="19" priority="16">
+      <formula>ROUND(D45,2-INT(LOG10(ABS(D45))))= ROUND(MIN($D45:$R45),2-INT(LOG10(ABS(MIN($D45:$R45)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D48:R48">
-    <cfRule type="top10" dxfId="18" priority="15" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="18" priority="15">
+      <formula>ROUND(D48,2-INT(LOG10(ABS(D48))))= ROUND(MIN($D48:$R48),2-INT(LOG10(ABS(MIN($D48:$R48)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D51:R51">
-    <cfRule type="top10" dxfId="17" priority="14" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="17" priority="14">
+      <formula>ROUND(D51,2-INT(LOG10(ABS(D51))))= ROUND(MIN($D51:$R51),2-INT(LOG10(ABS(MIN($D51:$R51)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D54:R54">
-    <cfRule type="top10" dxfId="16" priority="13" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="16" priority="13">
+      <formula>ROUND(D54,2-INT(LOG10(ABS(D54))))= ROUND(MIN($D54:$R54),2-INT(LOG10(ABS(MIN($D54:$R54)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D57:R57">
-    <cfRule type="top10" dxfId="15" priority="12" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="15" priority="12">
+      <formula>ROUND(D57,2-INT(LOG10(ABS(D57))))= ROUND(MIN($D57:$R57),2-INT(LOG10(ABS(MIN($D57:$R57)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D60:R60">
-    <cfRule type="top10" dxfId="14" priority="11" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>ROUND(D60,2-INT(LOG10(ABS(D60))))= ROUND(MIN($D60:$R60),2-INT(LOG10(ABS(MIN($D60:$R60)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D63:R63">
-    <cfRule type="top10" dxfId="13" priority="10" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="13" priority="10">
+      <formula>ROUND(D63,2-INT(LOG10(ABS(D63))))= ROUND(MIN($D63:$R63),2-INT(LOG10(ABS(MIN($D63:$R63)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D66:R66">
-    <cfRule type="top10" dxfId="12" priority="9" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="12" priority="9">
+      <formula>ROUND(D66,2-INT(LOG10(ABS(D66))))= ROUND(MIN($D66:$R66),2-INT(LOG10(ABS(MIN($D66:$R66)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:R69">
-    <cfRule type="top10" dxfId="11" priority="8" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="11" priority="8">
+      <formula>ROUND(D69,2-INT(LOG10(ABS(D69))))= ROUND(MIN($D69:$R69),2-INT(LOG10(ABS(MIN($D69:$R69)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D72:R72">
-    <cfRule type="top10" dxfId="10" priority="7" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="10" priority="7">
+      <formula>ROUND(D72,2-INT(LOG10(ABS(D72))))= ROUND(MIN($D72:$R72),2-INT(LOG10(ABS(MIN($D72:$R72)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D75:R75">
-    <cfRule type="top10" dxfId="9" priority="6" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="9" priority="6">
+      <formula>ROUND(D75,2-INT(LOG10(ABS(D75))))= ROUND(MIN($D75:$R75),2-INT(LOG10(ABS(MIN($D75:$R75)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D78:R78">
-    <cfRule type="top10" dxfId="8" priority="5" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="8" priority="5">
+      <formula>ROUND(D78,2-INT(LOG10(ABS(D78))))= ROUND(MIN($D78:$R78),2-INT(LOG10(ABS(MIN($D78:$R78)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D81:R81">
-    <cfRule type="top10" dxfId="7" priority="4" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="7" priority="4">
+      <formula>ROUND(D81,2-INT(LOG10(ABS(D81))))= ROUND(MIN($D81:$R81),2-INT(LOG10(ABS(MIN($D81:$R81)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D84:R84">
-    <cfRule type="top10" dxfId="6" priority="3" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>ROUND(D84,2-INT(LOG10(ABS(D84))))= ROUND(MIN($D84:$R84),2-INT(LOG10(ABS(MIN($D84:$R84)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D87:R87">
-    <cfRule type="top10" dxfId="5" priority="2" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>ROUND(D87,2-INT(LOG10(ABS(D87))))= ROUND(MIN($D87:$R87),2-INT(LOG10(ABS(MIN($D87:$R87)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D90:R90">
-    <cfRule type="top10" dxfId="4" priority="1" bottom="1" rank="1"/>
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>ROUND(D90,2-INT(LOG10(ABS(D90))))= ROUND(MIN($D90:$R90),2-INT(LOG10(ABS(MIN($D90:$R90)))))</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>